<commit_message>
ajustes nova versao; usando schema 3.3.0
</commit_message>
<xml_diff>
--- a/flask/app/static/examples/dcc_excel.xlsx
+++ b/flask/app/static/examples/dcc_excel.xlsx
@@ -85,7 +85,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -95,6 +95,9 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -18387,7 +18390,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:K6"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" style="1" min="1" max="1"/>
@@ -18797,44 +18800,56 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
-    <col width="21.5703125" customWidth="1" style="1" min="1" max="1"/>
-    <col width="31.7109375" customWidth="1" style="1" min="2" max="2"/>
-    <col width="10.42578125" customWidth="1" style="1" min="3" max="3"/>
-    <col width="23.85546875" customWidth="1" style="1" min="4" max="4"/>
-    <col width="13.140625" customWidth="1" style="1" min="5" max="5"/>
-    <col width="19.7109375" customWidth="1" style="1" min="6" max="6"/>
+    <col width="12" customWidth="1" style="1" min="1" max="1"/>
+    <col width="34" customWidth="1" style="1" min="2" max="2"/>
+    <col width="14" customWidth="1" style="1" min="3" max="3"/>
+    <col width="22" customWidth="1" style="1" min="4" max="4"/>
+    <col width="12" customWidth="1" style="1" min="5" max="5"/>
+    <col width="30" customWidth="1" style="1" min="6" max="6"/>
+    <col width="18" customWidth="1" style="1" min="7" max="7"/>
+    <col width="20" customWidth="1" style="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>label</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="5" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="5" t="inlineStr">
         <is>
           <t>col_name</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="5" t="inlineStr">
         <is>
           <t>unit</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="5" t="inlineStr">
         <is>
           <t>unc_relativa</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>relative_uncertainty_in_dcc</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>relative_unc_unit</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="inlineStr">
         <is>
           <t>refType</t>
         </is>
@@ -18862,6 +18877,11 @@
         </is>
       </c>
       <c r="E2" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
         <is>
           <t>Não</t>
         </is>

</xml_diff>